<commit_message>
Simplifie la fiche de suivi RA1 : plus sobre, sans date ni consigne
Retire la ligne de consigne et la ligne d'exemple pre-remplie
(date, nom, motif) demandees en trop par l'utilisateur. Garde une
mise en forme classique : titre fusionne en bandeau colore, en-tete
teinte, lignes vierges avec bandes alternees claires pour la
lisibilite. Toujours au format A3 portrait, ajuste sur une page.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01W7vxz49FDN6T7fNX2trwBJ
</commit_message>
<xml_diff>
--- a/Suivi_Zone_RA1_A3.xlsx
+++ b/Suivi_Zone_RA1_A3.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Suivi RA1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Suivi RA1'!$A$1:$D$39</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Suivi RA1'!$A$1:$D$38</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -30,32 +30,21 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <sz val="26"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <i val="1"/>
-      <color rgb="00444444"/>
-      <sz val="12"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="24"/>
     </font>
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="14"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <i val="1"/>
-      <color rgb="007A6A00"/>
-      <sz val="11"/>
+      <color rgb="001F3864"/>
+      <sz val="13"/>
     </font>
     <font>
       <name val="Arial"/>
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -64,12 +53,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F2937"/>
+        <fgColor rgb="002E4E7E"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF7CC"/>
+        <fgColor rgb="00BDD0EA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F5FA"/>
       </patternFill>
     </fill>
   </fills>
@@ -83,37 +77,34 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00000000"/>
+        <color rgb="00B7C3D0"/>
       </left>
       <right style="thin">
-        <color rgb="00000000"/>
+        <color rgb="00B7C3D0"/>
       </right>
       <top style="thin">
-        <color rgb="00000000"/>
+        <color rgb="00B7C3D0"/>
       </top>
       <bottom style="thin">
-        <color rgb="00000000"/>
+        <color rgb="00B7C3D0"/>
       </bottom>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -481,7 +472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D39"/>
+  <dimension ref="A1:D38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -490,273 +481,254 @@
     <col width="90" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1" ht="42" customHeight="1">
+    <row r="1" ht="40" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>ZONE RA1 — FICHE DE SUIVI</t>
+          <t>ZONE RA1  —  FICHE DE SUIVI</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="20" customHeight="1">
+    <row r="2" ht="26" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>A remplir au stylo par le cariste a chaque mouvement / intervention sur la zone</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="8" customHeight="1"/>
-    <row r="4" ht="26" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>Qui</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>UM</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>Raison</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="22" customHeight="1">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>20/08/2026</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>Exemple : J. Dupont</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>Exemple : palette abimee deplacee en zone controle qualite</t>
-        </is>
-      </c>
+    <row r="3" ht="24" customHeight="1">
+      <c r="A3" s="3" t="inlineStr"/>
+      <c r="B3" s="3" t="inlineStr"/>
+      <c r="C3" s="3" t="inlineStr"/>
+      <c r="D3" s="3" t="inlineStr"/>
+    </row>
+    <row r="4" ht="24" customHeight="1">
+      <c r="A4" s="4" t="inlineStr"/>
+      <c r="B4" s="4" t="inlineStr"/>
+      <c r="C4" s="4" t="inlineStr"/>
+      <c r="D4" s="4" t="inlineStr"/>
+    </row>
+    <row r="5" ht="24" customHeight="1">
+      <c r="A5" s="3" t="inlineStr"/>
+      <c r="B5" s="3" t="inlineStr"/>
+      <c r="C5" s="3" t="inlineStr"/>
+      <c r="D5" s="3" t="inlineStr"/>
     </row>
     <row r="6" ht="24" customHeight="1">
-      <c r="A6" s="5" t="inlineStr"/>
-      <c r="B6" s="5" t="inlineStr"/>
-      <c r="C6" s="5" t="inlineStr"/>
-      <c r="D6" s="5" t="inlineStr"/>
+      <c r="A6" s="4" t="inlineStr"/>
+      <c r="B6" s="4" t="inlineStr"/>
+      <c r="C6" s="4" t="inlineStr"/>
+      <c r="D6" s="4" t="inlineStr"/>
     </row>
     <row r="7" ht="24" customHeight="1">
-      <c r="A7" s="5" t="inlineStr"/>
-      <c r="B7" s="5" t="inlineStr"/>
-      <c r="C7" s="5" t="inlineStr"/>
-      <c r="D7" s="5" t="inlineStr"/>
+      <c r="A7" s="3" t="inlineStr"/>
+      <c r="B7" s="3" t="inlineStr"/>
+      <c r="C7" s="3" t="inlineStr"/>
+      <c r="D7" s="3" t="inlineStr"/>
     </row>
     <row r="8" ht="24" customHeight="1">
-      <c r="A8" s="5" t="inlineStr"/>
-      <c r="B8" s="5" t="inlineStr"/>
-      <c r="C8" s="5" t="inlineStr"/>
-      <c r="D8" s="5" t="inlineStr"/>
+      <c r="A8" s="4" t="inlineStr"/>
+      <c r="B8" s="4" t="inlineStr"/>
+      <c r="C8" s="4" t="inlineStr"/>
+      <c r="D8" s="4" t="inlineStr"/>
     </row>
     <row r="9" ht="24" customHeight="1">
-      <c r="A9" s="5" t="inlineStr"/>
-      <c r="B9" s="5" t="inlineStr"/>
-      <c r="C9" s="5" t="inlineStr"/>
-      <c r="D9" s="5" t="inlineStr"/>
+      <c r="A9" s="3" t="inlineStr"/>
+      <c r="B9" s="3" t="inlineStr"/>
+      <c r="C9" s="3" t="inlineStr"/>
+      <c r="D9" s="3" t="inlineStr"/>
     </row>
     <row r="10" ht="24" customHeight="1">
-      <c r="A10" s="5" t="inlineStr"/>
-      <c r="B10" s="5" t="inlineStr"/>
-      <c r="C10" s="5" t="inlineStr"/>
-      <c r="D10" s="5" t="inlineStr"/>
+      <c r="A10" s="4" t="inlineStr"/>
+      <c r="B10" s="4" t="inlineStr"/>
+      <c r="C10" s="4" t="inlineStr"/>
+      <c r="D10" s="4" t="inlineStr"/>
     </row>
     <row r="11" ht="24" customHeight="1">
-      <c r="A11" s="5" t="inlineStr"/>
-      <c r="B11" s="5" t="inlineStr"/>
-      <c r="C11" s="5" t="inlineStr"/>
-      <c r="D11" s="5" t="inlineStr"/>
+      <c r="A11" s="3" t="inlineStr"/>
+      <c r="B11" s="3" t="inlineStr"/>
+      <c r="C11" s="3" t="inlineStr"/>
+      <c r="D11" s="3" t="inlineStr"/>
     </row>
     <row r="12" ht="24" customHeight="1">
-      <c r="A12" s="5" t="inlineStr"/>
-      <c r="B12" s="5" t="inlineStr"/>
-      <c r="C12" s="5" t="inlineStr"/>
-      <c r="D12" s="5" t="inlineStr"/>
+      <c r="A12" s="4" t="inlineStr"/>
+      <c r="B12" s="4" t="inlineStr"/>
+      <c r="C12" s="4" t="inlineStr"/>
+      <c r="D12" s="4" t="inlineStr"/>
     </row>
     <row r="13" ht="24" customHeight="1">
-      <c r="A13" s="5" t="inlineStr"/>
-      <c r="B13" s="5" t="inlineStr"/>
-      <c r="C13" s="5" t="inlineStr"/>
-      <c r="D13" s="5" t="inlineStr"/>
+      <c r="A13" s="3" t="inlineStr"/>
+      <c r="B13" s="3" t="inlineStr"/>
+      <c r="C13" s="3" t="inlineStr"/>
+      <c r="D13" s="3" t="inlineStr"/>
     </row>
     <row r="14" ht="24" customHeight="1">
-      <c r="A14" s="5" t="inlineStr"/>
-      <c r="B14" s="5" t="inlineStr"/>
-      <c r="C14" s="5" t="inlineStr"/>
-      <c r="D14" s="5" t="inlineStr"/>
+      <c r="A14" s="4" t="inlineStr"/>
+      <c r="B14" s="4" t="inlineStr"/>
+      <c r="C14" s="4" t="inlineStr"/>
+      <c r="D14" s="4" t="inlineStr"/>
     </row>
     <row r="15" ht="24" customHeight="1">
-      <c r="A15" s="5" t="inlineStr"/>
-      <c r="B15" s="5" t="inlineStr"/>
-      <c r="C15" s="5" t="inlineStr"/>
-      <c r="D15" s="5" t="inlineStr"/>
+      <c r="A15" s="3" t="inlineStr"/>
+      <c r="B15" s="3" t="inlineStr"/>
+      <c r="C15" s="3" t="inlineStr"/>
+      <c r="D15" s="3" t="inlineStr"/>
     </row>
     <row r="16" ht="24" customHeight="1">
-      <c r="A16" s="5" t="inlineStr"/>
-      <c r="B16" s="5" t="inlineStr"/>
-      <c r="C16" s="5" t="inlineStr"/>
-      <c r="D16" s="5" t="inlineStr"/>
+      <c r="A16" s="4" t="inlineStr"/>
+      <c r="B16" s="4" t="inlineStr"/>
+      <c r="C16" s="4" t="inlineStr"/>
+      <c r="D16" s="4" t="inlineStr"/>
     </row>
     <row r="17" ht="24" customHeight="1">
-      <c r="A17" s="5" t="inlineStr"/>
-      <c r="B17" s="5" t="inlineStr"/>
-      <c r="C17" s="5" t="inlineStr"/>
-      <c r="D17" s="5" t="inlineStr"/>
+      <c r="A17" s="3" t="inlineStr"/>
+      <c r="B17" s="3" t="inlineStr"/>
+      <c r="C17" s="3" t="inlineStr"/>
+      <c r="D17" s="3" t="inlineStr"/>
     </row>
     <row r="18" ht="24" customHeight="1">
-      <c r="A18" s="5" t="inlineStr"/>
-      <c r="B18" s="5" t="inlineStr"/>
-      <c r="C18" s="5" t="inlineStr"/>
-      <c r="D18" s="5" t="inlineStr"/>
+      <c r="A18" s="4" t="inlineStr"/>
+      <c r="B18" s="4" t="inlineStr"/>
+      <c r="C18" s="4" t="inlineStr"/>
+      <c r="D18" s="4" t="inlineStr"/>
     </row>
     <row r="19" ht="24" customHeight="1">
-      <c r="A19" s="5" t="inlineStr"/>
-      <c r="B19" s="5" t="inlineStr"/>
-      <c r="C19" s="5" t="inlineStr"/>
-      <c r="D19" s="5" t="inlineStr"/>
+      <c r="A19" s="3" t="inlineStr"/>
+      <c r="B19" s="3" t="inlineStr"/>
+      <c r="C19" s="3" t="inlineStr"/>
+      <c r="D19" s="3" t="inlineStr"/>
     </row>
     <row r="20" ht="24" customHeight="1">
-      <c r="A20" s="5" t="inlineStr"/>
-      <c r="B20" s="5" t="inlineStr"/>
-      <c r="C20" s="5" t="inlineStr"/>
-      <c r="D20" s="5" t="inlineStr"/>
+      <c r="A20" s="4" t="inlineStr"/>
+      <c r="B20" s="4" t="inlineStr"/>
+      <c r="C20" s="4" t="inlineStr"/>
+      <c r="D20" s="4" t="inlineStr"/>
     </row>
     <row r="21" ht="24" customHeight="1">
-      <c r="A21" s="5" t="inlineStr"/>
-      <c r="B21" s="5" t="inlineStr"/>
-      <c r="C21" s="5" t="inlineStr"/>
-      <c r="D21" s="5" t="inlineStr"/>
+      <c r="A21" s="3" t="inlineStr"/>
+      <c r="B21" s="3" t="inlineStr"/>
+      <c r="C21" s="3" t="inlineStr"/>
+      <c r="D21" s="3" t="inlineStr"/>
     </row>
     <row r="22" ht="24" customHeight="1">
-      <c r="A22" s="5" t="inlineStr"/>
-      <c r="B22" s="5" t="inlineStr"/>
-      <c r="C22" s="5" t="inlineStr"/>
-      <c r="D22" s="5" t="inlineStr"/>
+      <c r="A22" s="4" t="inlineStr"/>
+      <c r="B22" s="4" t="inlineStr"/>
+      <c r="C22" s="4" t="inlineStr"/>
+      <c r="D22" s="4" t="inlineStr"/>
     </row>
     <row r="23" ht="24" customHeight="1">
-      <c r="A23" s="5" t="inlineStr"/>
-      <c r="B23" s="5" t="inlineStr"/>
-      <c r="C23" s="5" t="inlineStr"/>
-      <c r="D23" s="5" t="inlineStr"/>
+      <c r="A23" s="3" t="inlineStr"/>
+      <c r="B23" s="3" t="inlineStr"/>
+      <c r="C23" s="3" t="inlineStr"/>
+      <c r="D23" s="3" t="inlineStr"/>
     </row>
     <row r="24" ht="24" customHeight="1">
-      <c r="A24" s="5" t="inlineStr"/>
-      <c r="B24" s="5" t="inlineStr"/>
-      <c r="C24" s="5" t="inlineStr"/>
-      <c r="D24" s="5" t="inlineStr"/>
+      <c r="A24" s="4" t="inlineStr"/>
+      <c r="B24" s="4" t="inlineStr"/>
+      <c r="C24" s="4" t="inlineStr"/>
+      <c r="D24" s="4" t="inlineStr"/>
     </row>
     <row r="25" ht="24" customHeight="1">
-      <c r="A25" s="5" t="inlineStr"/>
-      <c r="B25" s="5" t="inlineStr"/>
-      <c r="C25" s="5" t="inlineStr"/>
-      <c r="D25" s="5" t="inlineStr"/>
+      <c r="A25" s="3" t="inlineStr"/>
+      <c r="B25" s="3" t="inlineStr"/>
+      <c r="C25" s="3" t="inlineStr"/>
+      <c r="D25" s="3" t="inlineStr"/>
     </row>
     <row r="26" ht="24" customHeight="1">
-      <c r="A26" s="5" t="inlineStr"/>
-      <c r="B26" s="5" t="inlineStr"/>
-      <c r="C26" s="5" t="inlineStr"/>
-      <c r="D26" s="5" t="inlineStr"/>
+      <c r="A26" s="4" t="inlineStr"/>
+      <c r="B26" s="4" t="inlineStr"/>
+      <c r="C26" s="4" t="inlineStr"/>
+      <c r="D26" s="4" t="inlineStr"/>
     </row>
     <row r="27" ht="24" customHeight="1">
-      <c r="A27" s="5" t="inlineStr"/>
-      <c r="B27" s="5" t="inlineStr"/>
-      <c r="C27" s="5" t="inlineStr"/>
-      <c r="D27" s="5" t="inlineStr"/>
+      <c r="A27" s="3" t="inlineStr"/>
+      <c r="B27" s="3" t="inlineStr"/>
+      <c r="C27" s="3" t="inlineStr"/>
+      <c r="D27" s="3" t="inlineStr"/>
     </row>
     <row r="28" ht="24" customHeight="1">
-      <c r="A28" s="5" t="inlineStr"/>
-      <c r="B28" s="5" t="inlineStr"/>
-      <c r="C28" s="5" t="inlineStr"/>
-      <c r="D28" s="5" t="inlineStr"/>
+      <c r="A28" s="4" t="inlineStr"/>
+      <c r="B28" s="4" t="inlineStr"/>
+      <c r="C28" s="4" t="inlineStr"/>
+      <c r="D28" s="4" t="inlineStr"/>
     </row>
     <row r="29" ht="24" customHeight="1">
-      <c r="A29" s="5" t="inlineStr"/>
-      <c r="B29" s="5" t="inlineStr"/>
-      <c r="C29" s="5" t="inlineStr"/>
-      <c r="D29" s="5" t="inlineStr"/>
+      <c r="A29" s="3" t="inlineStr"/>
+      <c r="B29" s="3" t="inlineStr"/>
+      <c r="C29" s="3" t="inlineStr"/>
+      <c r="D29" s="3" t="inlineStr"/>
     </row>
     <row r="30" ht="24" customHeight="1">
-      <c r="A30" s="5" t="inlineStr"/>
-      <c r="B30" s="5" t="inlineStr"/>
-      <c r="C30" s="5" t="inlineStr"/>
-      <c r="D30" s="5" t="inlineStr"/>
+      <c r="A30" s="4" t="inlineStr"/>
+      <c r="B30" s="4" t="inlineStr"/>
+      <c r="C30" s="4" t="inlineStr"/>
+      <c r="D30" s="4" t="inlineStr"/>
     </row>
     <row r="31" ht="24" customHeight="1">
-      <c r="A31" s="5" t="inlineStr"/>
-      <c r="B31" s="5" t="inlineStr"/>
-      <c r="C31" s="5" t="inlineStr"/>
-      <c r="D31" s="5" t="inlineStr"/>
+      <c r="A31" s="3" t="inlineStr"/>
+      <c r="B31" s="3" t="inlineStr"/>
+      <c r="C31" s="3" t="inlineStr"/>
+      <c r="D31" s="3" t="inlineStr"/>
     </row>
     <row r="32" ht="24" customHeight="1">
-      <c r="A32" s="5" t="inlineStr"/>
-      <c r="B32" s="5" t="inlineStr"/>
-      <c r="C32" s="5" t="inlineStr"/>
-      <c r="D32" s="5" t="inlineStr"/>
+      <c r="A32" s="4" t="inlineStr"/>
+      <c r="B32" s="4" t="inlineStr"/>
+      <c r="C32" s="4" t="inlineStr"/>
+      <c r="D32" s="4" t="inlineStr"/>
     </row>
     <row r="33" ht="24" customHeight="1">
-      <c r="A33" s="5" t="inlineStr"/>
-      <c r="B33" s="5" t="inlineStr"/>
-      <c r="C33" s="5" t="inlineStr"/>
-      <c r="D33" s="5" t="inlineStr"/>
+      <c r="A33" s="3" t="inlineStr"/>
+      <c r="B33" s="3" t="inlineStr"/>
+      <c r="C33" s="3" t="inlineStr"/>
+      <c r="D33" s="3" t="inlineStr"/>
     </row>
     <row r="34" ht="24" customHeight="1">
-      <c r="A34" s="5" t="inlineStr"/>
-      <c r="B34" s="5" t="inlineStr"/>
-      <c r="C34" s="5" t="inlineStr"/>
-      <c r="D34" s="5" t="inlineStr"/>
+      <c r="A34" s="4" t="inlineStr"/>
+      <c r="B34" s="4" t="inlineStr"/>
+      <c r="C34" s="4" t="inlineStr"/>
+      <c r="D34" s="4" t="inlineStr"/>
     </row>
     <row r="35" ht="24" customHeight="1">
-      <c r="A35" s="5" t="inlineStr"/>
-      <c r="B35" s="5" t="inlineStr"/>
-      <c r="C35" s="5" t="inlineStr"/>
-      <c r="D35" s="5" t="inlineStr"/>
+      <c r="A35" s="3" t="inlineStr"/>
+      <c r="B35" s="3" t="inlineStr"/>
+      <c r="C35" s="3" t="inlineStr"/>
+      <c r="D35" s="3" t="inlineStr"/>
     </row>
     <row r="36" ht="24" customHeight="1">
-      <c r="A36" s="5" t="inlineStr"/>
-      <c r="B36" s="5" t="inlineStr"/>
-      <c r="C36" s="5" t="inlineStr"/>
-      <c r="D36" s="5" t="inlineStr"/>
+      <c r="A36" s="4" t="inlineStr"/>
+      <c r="B36" s="4" t="inlineStr"/>
+      <c r="C36" s="4" t="inlineStr"/>
+      <c r="D36" s="4" t="inlineStr"/>
     </row>
     <row r="37" ht="24" customHeight="1">
-      <c r="A37" s="5" t="inlineStr"/>
-      <c r="B37" s="5" t="inlineStr"/>
-      <c r="C37" s="5" t="inlineStr"/>
-      <c r="D37" s="5" t="inlineStr"/>
+      <c r="A37" s="3" t="inlineStr"/>
+      <c r="B37" s="3" t="inlineStr"/>
+      <c r="C37" s="3" t="inlineStr"/>
+      <c r="D37" s="3" t="inlineStr"/>
     </row>
     <row r="38" ht="24" customHeight="1">
-      <c r="A38" s="5" t="inlineStr"/>
-      <c r="B38" s="5" t="inlineStr"/>
-      <c r="C38" s="5" t="inlineStr"/>
-      <c r="D38" s="5" t="inlineStr"/>
-    </row>
-    <row r="39" ht="24" customHeight="1">
-      <c r="A39" s="5" t="inlineStr"/>
-      <c r="B39" s="5" t="inlineStr"/>
-      <c r="C39" s="5" t="inlineStr"/>
-      <c r="D39" s="5" t="inlineStr"/>
+      <c r="A38" s="4" t="inlineStr"/>
+      <c r="B38" s="4" t="inlineStr"/>
+      <c r="C38" s="4" t="inlineStr"/>
+      <c r="D38" s="4" t="inlineStr"/>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="1">
     <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A2:D2"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.5" right="0.5" top="0.6" bottom="0.6" header="0.2" footer="0.2"/>

</xml_diff>

<commit_message>
Elargit les colonnes UM et Raison de la fiche de suivi RA1
Reduit legerement Date/Qui et elargit UM (12 -> 20) et Raison
(90 -> 115) pour laisser plus de place a l'ecriture manuscrite.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01W7vxz49FDN6T7fNX2trwBJ
</commit_message>
<xml_diff>
--- a/Suivi_Zone_RA1_A3.xlsx
+++ b/Suivi_Zone_RA1_A3.xlsx
@@ -475,10 +475,10 @@
   <dimension ref="A1:D38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="90" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="115" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1" ht="40" customHeight="1">

</xml_diff>